<commit_message>
Fill HSK2 parts 3 (ID 601-650) with parts of speech
</commit_message>
<xml_diff>
--- a/HSK2_parts_of_speech_3(601-650).xlsx
+++ b/HSK2_parts_of_speech_3(601-650).xlsx
@@ -85,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -97,6 +97,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -644,6 +647,26 @@
           <t>пояс</t>
         </is>
       </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>ремень, пояс; лента</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>носить (на себе); приводить (带朋友来); приносить (带东西)</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>для лент и полос (一条带子)</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>离合-подобное: 带...了 (带了本书)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -670,6 +693,16 @@
           <t>нести с собой</t>
         </is>
       </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>приносить с собой; приводить (с собой)</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>глагол + направленное дополнение (带来 = 带+来), цельная глагольная конструкция</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -696,6 +729,16 @@
           <t>организация</t>
         </is>
       </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>единица; организация, предприятие; воинская часть; единица измерения</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>единичный, одиночный (单位数)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -722,6 +765,16 @@
           <t>но</t>
         </is>
       </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>лишь, только (不但...不...)</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>но, однако</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -748,6 +801,11 @@
           <t>но</t>
         </is>
       </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>но, однако</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -774,6 +832,11 @@
           <t>яйцо</t>
         </is>
       </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>яйцо; яичко (разг.)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -800,6 +863,26 @@
           <t>равняться, являться</t>
         </is>
       </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>быть, являться; служить (当老师); совпадать (正当...)</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>как раз, именно (当时)</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>в качестве, в роли (当作); когда (当他回来时)</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>многозначный; предложное употребление 当...时</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -826,6 +909,21 @@
           <t>в то время</t>
         </is>
       </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>то время</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>тогда, в то время</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr">
+        <is>
+          <t>тогдашний, прежний (当时的情况)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -852,6 +950,26 @@
           <t>упасть, повалиться</t>
         </is>
       </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>упасть, повалиться; терпеть неудачу (倒台)</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>все-таки, наоборот (反而倒)</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>усилит. частица (好倒好，可是...)</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>полифония dǎo/dào; здесь чтение dǎo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -878,6 +996,16 @@
           <t>везде</t>
         </is>
       </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>место, повсюду</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>везде, повсюду</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -904,6 +1032,26 @@
           <t>перевернуть</t>
         </is>
       </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>переворачивать; опрокидывать; наливать (倒茶); отлить (倒垃圾)</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>наоборот, вопреки ожиданию (反倒); все же (他倒是来了)</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>已达程度 (好倒了 — устар.)</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>чтение dào; многозначный</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -930,6 +1078,26 @@
           <t>путь, дорога</t>
         </is>
       </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>дорога, путь; направление; принцип (道理)</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>говорить, произносить (道谢, 说长道短)</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>для длинных узких предметов и абстрактных путей (一道河, 一道题, 一道门)</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>искусственный (道貌岸然)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -956,6 +1124,16 @@
           <t>истина, суть</t>
         </is>
       </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>истина, здравый смысл; причина, логика</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="inlineStr">
+        <is>
+          <t>составное существительное 道+理</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -982,6 +1160,11 @@
           <t>путь, полотно дороги</t>
         </is>
       </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>дорога, путь (в прямом и переносном смысле)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1008,6 +1191,26 @@
           <t>получать, добывать</t>
         </is>
       </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>получать, добывать; достичь (得奖)</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>надо, необходимо (dé: 得去)</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>полифония: dé получать / děн must / de частица; ID 615 — чтение dé</t>
+        </is>
+      </c>
+      <c r="Y16" s="5" t="inlineStr">
+        <is>
+          <t>в значении «надо» читается děн</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1034,6 +1237,16 @@
           <t>получить в результате</t>
         </is>
       </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>получить (вывод); сделать (заключение)</t>
+        </is>
+      </c>
+      <c r="X17" s="5" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение (得出 = 得+出)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1060,6 +1273,21 @@
           <t>если</t>
         </is>
       </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>слова, речь (在...的情况下)</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>если (в конце условия: 你要是不去的话)</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>условная частица 的话; также существительное 话 в составе</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1086,6 +1314,21 @@
           <t>частица, используемая после глагола для описания действия</t>
         </is>
       </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>структурная частица после глагола для описания действия/дополнения степени (跑得快)</t>
+        </is>
+      </c>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>частица de (中性), не самостоятельное слово</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1112,6 +1355,21 @@
           <t>лампа</t>
         </is>
       </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>лампа, светильник; огонь (灯火)</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>для ламп и фонарей (一盏灯) — само как счётное нет</t>
+        </is>
+      </c>
+      <c r="X20" s="5" t="inlineStr">
+        <is>
+          <t>существительное; часто в сочетаниях 关灯/开灯/点灯</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1138,6 +1396,36 @@
           <t>и т.д., и др.</t>
         </is>
       </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>ранг, категория (等级)</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>ждать, ожидать (等人); равняться, быть равным (=等于)</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>для классов/рангов (一等舱)</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>равняться, быть равным (=等于)</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>перечисление «и т.д.» (桌椅板凳等)</t>
+        </is>
+      </c>
+      <c r="X21" s="5" t="inlineStr">
+        <is>
+          <t>多义</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1164,6 +1452,16 @@
           <t>ждать до...</t>
         </is>
       </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>ждать до (какого-то момента)</t>
+        </is>
+      </c>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>глагол 等 + результативное дополнение 到</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1190,6 +1488,16 @@
           <t>равно, быть равным</t>
         </is>
       </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>равняться, быть равным; соответствовать</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>то есть, равно как</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1216,6 +1524,21 @@
           <t>низкий</t>
         </is>
       </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>понижать, склонять (低头)</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>низкий (低矮); дешёвый (价格低); низкий (по уровню)</t>
+        </is>
+      </c>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>низкий (низкочастотный)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1242,6 +1565,21 @@
           <t>Земля</t>
         </is>
       </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Земля (планета)</t>
+        </is>
+      </c>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>земной, глобальный (地球人)</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="inlineStr">
+        <is>
+          <t>составное: 地 (земля) + 球 (шар)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1268,6 +1606,16 @@
           <t>метро</t>
         </is>
       </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>метро, подземка</t>
+        </is>
+      </c>
+      <c r="X26" s="5" t="inlineStr">
+        <is>
+          <t>сокращение от 地下铁路</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1294,6 +1642,16 @@
           <t>станция метро</t>
         </is>
       </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>станция метро</t>
+        </is>
+      </c>
+      <c r="X27" s="5" t="inlineStr">
+        <is>
+          <t>словосочетание 地铁+站, устойчивое название</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1320,6 +1678,16 @@
           <t>кивать</t>
         </is>
       </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>кивать (головкой)</t>
+        </is>
+      </c>
+      <c r="X28" s="5" t="inlineStr">
+        <is>
+          <t>离合词 (点了个头): глагол 点 + объект 头</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1346,6 +1714,16 @@
           <t>магазин</t>
         </is>
       </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>магазин, лавка; ресторан; гостиница (旅店)</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>для магазинов (一家店)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1372,6 +1750,21 @@
           <t>падать</t>
         </is>
       </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>падать, упасть; терять (丢); исчезать (消失掉)</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr">
+        <is>
+          <t>частично грамматализуется как результативное дополнение (吃掉, 扔掉)</t>
+        </is>
+      </c>
+      <c r="X30" s="5" t="inlineStr">
+        <is>
+          <t>полифония diào/dāo; здесь diào — падать; как дополнение потери (丢失掉)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1398,6 +1791,16 @@
           <t>северо-восток</t>
         </is>
       </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>северо-восток; Северо-Восточный Китай (Дунбэй)</t>
+        </is>
+      </c>
+      <c r="W31" s="5" t="inlineStr">
+        <is>
+          <t>северо-восточный (东北风)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1424,6 +1827,21 @@
           <t>восток</t>
         </is>
       </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>восток; Восток (东方文化)</t>
+        </is>
+      </c>
+      <c r="W32" s="5" t="inlineStr">
+        <is>
+          <t>восточный (东方人)</t>
+        </is>
+      </c>
+      <c r="X32" s="5" t="inlineStr">
+        <is>
+          <t>составное 东+方</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1450,6 +1868,21 @@
           <t>юго-восток</t>
         </is>
       </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>юго-восток</t>
+        </is>
+      </c>
+      <c r="W33" s="5" t="inlineStr">
+        <is>
+          <t>юго-восточный (东南方向)</t>
+        </is>
+      </c>
+      <c r="X33" s="5" t="inlineStr">
+        <is>
+          <t>составное 东+南</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1476,6 +1909,21 @@
           <t>зима</t>
         </is>
       </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>зима</t>
+        </is>
+      </c>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>зимний (冬天里的事)</t>
+        </is>
+      </c>
+      <c r="X34" s="5" t="inlineStr">
+        <is>
+          <t>составное 冬+天 (временное слово)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1502,6 +1950,11 @@
           <t>понимать</t>
         </is>
       </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>понимать, соображать (懂中文)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1528,6 +1981,16 @@
           <t>понимать, разбираться</t>
         </is>
       </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>понимать, разбираться (更深)</t>
+        </is>
+      </c>
+      <c r="X36" s="5" t="inlineStr">
+        <is>
+          <t>глагол 懂 + аспект-частица 得 (可能/результат)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1554,6 +2017,16 @@
           <t>животное</t>
         </is>
       </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>животное</t>
+        </is>
+      </c>
+      <c r="W37" s="5" t="inlineStr">
+        <is>
+          <t>животный (动物世界)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1580,6 +2053,16 @@
           <t>зоопарк</t>
         </is>
       </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>зоопарк</t>
+        </is>
+      </c>
+      <c r="X38" s="5" t="inlineStr">
+        <is>
+          <t>составное 动物园</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1606,6 +2089,16 @@
           <t>произношение</t>
         </is>
       </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>произношение, чтение (读音准确)</t>
+        </is>
+      </c>
+      <c r="X39" s="5" t="inlineStr">
+        <is>
+          <t>составное 读+音</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1632,6 +2125,26 @@
           <t>градус</t>
         </is>
       </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>градус; температура; степень; год (年度)</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>мерить, проходить (度过假期)</t>
+        </is>
+      </c>
+      <c r="O40" s="5" t="inlineStr">
+        <is>
+          <t>для градусов и повторяемости событий (一度火, 两度访问)</t>
+        </is>
+      </c>
+      <c r="X40" s="5" t="inlineStr">
+        <is>
+          <t>多义</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1658,6 +2171,26 @@
           <t>короткий</t>
         </is>
       </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>укорачивать (缩短)</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>короткий (长度/时间); краткий</t>
+        </is>
+      </c>
+      <c r="W41" s="5" t="inlineStr">
+        <is>
+          <t>короткий (短篇小说)</t>
+        </is>
+      </c>
+      <c r="X41" s="5" t="inlineStr">
+        <is>
+          <t>часто в парах 长短</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1684,6 +2217,16 @@
           <t>короткое сообщение</t>
         </is>
       </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>SMS, короткое сообщение</t>
+        </is>
+      </c>
+      <c r="X42" s="5" t="inlineStr">
+        <is>
+          <t>составное 短+信</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1710,6 +2253,21 @@
           <t>отрезок, абзац</t>
         </is>
       </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>отрезок, фрагмент; раздел</t>
+        </is>
+      </c>
+      <c r="O43" s="5" t="inlineStr">
+        <is>
+          <t>для отрезков, частей, абзацев (一段路, 一段时间, 两段代码)</t>
+        </is>
+      </c>
+      <c r="W43" s="5" t="inlineStr">
+        <is>
+          <t>сегментный (段落)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1736,6 +2294,26 @@
           <t>команда</t>
         </is>
       </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>команда, отряд; очередь (排队)</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>объединяться в группу (队队相连) — редко</t>
+        </is>
+      </c>
+      <c r="O44" s="5" t="inlineStr">
+        <is>
+          <t>для команд/отрядов (一队人)</t>
+        </is>
+      </c>
+      <c r="X44" s="5" t="inlineStr">
+        <is>
+          <t>в осн. сущ./кл.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1762,6 +2340,21 @@
           <t>лидер, капитан</t>
         </is>
       </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>начальник команды, капитан</t>
+        </is>
+      </c>
+      <c r="W45" s="5" t="inlineStr">
+        <is>
+          <t>командирский (队长级别)</t>
+        </is>
+      </c>
+      <c r="X45" s="5" t="inlineStr">
+        <is>
+          <t>составное 队+长 (cháng)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1788,6 +2381,46 @@
           <t>по отношению к, о, по; относиться к...</t>
         </is>
       </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>пара; противная сторона (对手)</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>относиться, обрабатывать (对付); сверять (对答案)</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>правильный, верный (对不对)</t>
+        </is>
+      </c>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>для пар (一对夫妻)</t>
+        </is>
+      </c>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>вместе, взаимно (对望)</t>
+        </is>
+      </c>
+      <c r="R46" s="5" t="inlineStr">
+        <is>
+          <t>по отношению к, насчёт (对我很好)</t>
+        </is>
+      </c>
+      <c r="W46" s="5" t="inlineStr">
+        <is>
+          <t>парный, анти-</t>
+        </is>
+      </c>
+      <c r="X46" s="5" t="inlineStr">
+        <is>
+          <t>крайне многозначный</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1814,6 +2447,21 @@
           <t>диалог</t>
         </is>
       </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>диалог; переговоры (进行对话)</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>вести диалог (对话交流)</t>
+        </is>
+      </c>
+      <c r="X47" s="5" t="inlineStr">
+        <is>
+          <t>离合-подобное 对+话</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1840,6 +2488,31 @@
           <t>напротив</t>
         </is>
       </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>противоположная сторона (对面是银行)</t>
+        </is>
+      </c>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>напротив, face-to-face (面对面)</t>
+        </is>
+      </c>
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>навстречу, напротив (对面走来)</t>
+        </is>
+      </c>
+      <c r="W48" s="5" t="inlineStr">
+        <is>
+          <t>противоположный</t>
+        </is>
+      </c>
+      <c r="X48" s="5" t="inlineStr">
+        <is>
+          <t>локативная конструкция 对+面</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1866,6 +2539,31 @@
           <t>побольше</t>
         </is>
       </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>превышать (多余); хвалить (夸多)</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>многий, многочисленный (人多)</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>несколько (十多天)</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>сколько (多少钱); насколько (多好!)</t>
+        </is>
+      </c>
+      <c r="X49" s="5" t="inlineStr">
+        <is>
+          <t>多义</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1892,6 +2590,21 @@
           <t>как давно</t>
         </is>
       </c>
+      <c r="P50" s="5" t="inlineStr">
+        <is>
+          <t>как долго? сколько времени?</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>как давно? (你多久没见他了?)</t>
+        </is>
+      </c>
+      <c r="X50" s="5" t="inlineStr">
+        <is>
+          <t>вопросительная конструкция 多+久</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1916,6 +2629,16 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>насколько</t>
+        </is>
+      </c>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>насколько, как (多么好!); в какой степени</t>
+        </is>
+      </c>
+      <c r="X51" s="5" t="inlineStr">
+        <is>
+          <t>вопросительно-восклицательное наречие</t>
         </is>
       </c>
     </row>

</xml_diff>